<commit_message>
Version Dataverse second pass workbench
</commit_message>
<xml_diff>
--- a/outputs/control_operativo_20260615/control_operativo.xlsx
+++ b/outputs/control_operativo_20260615/control_operativo.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R38e155c72def401a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro" sheetId="2" r:id="R8d0519fe008143a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertas" sheetId="3" r:id="R7eedd83a13a4431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" r:id="Rd589f873a1f44824"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rfc5667e7748a4b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro" sheetId="2" r:id="Rd2e7ee0fe8ad4cba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertas" sheetId="3" r:id="Rf384183da1cd45b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" r:id="R69586ed265fc4162"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DeltasTable" displayName="DeltasTable" ref="A5:J65" headerRowCount="1">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DeltasTable" displayName="DeltasTable" ref="A5:O65" headerRowCount="1">
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="Delta"/>
     <x:tableColumn id="2" name="Fecha"/>
     <x:tableColumn id="3" name="Superficie"/>
@@ -190,6 +190,11 @@
     <x:tableColumn id="8" name="Salida"/>
     <x:tableColumn id="9" name="Hito"/>
     <x:tableColumn id="10" name="Notas"/>
+    <x:tableColumn id="11" name="Dataverse estado"/>
+    <x:tableColumn id="12" name="Ambiente"/>
+    <x:tableColumn id="13" name="Target exacto"/>
+    <x:tableColumn id="14" name="Gate live"/>
+    <x:tableColumn id="15" name="Postcheck"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -536,7 +541,7 @@
       </x:c>
       <x:c r="B11" s="10" t="n">
         <x:f>COUNTIF(Alertas!$B$6:$B$35,"Alta")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D11" s="7"/>
       <x:c r="E11" s="7"/>
@@ -579,10 +584,15 @@
     <x:col min="5" max="5" width="16.25" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="16.25" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16.25" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="37.5" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="37.5" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="37.5" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="27.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -598,6 +608,11 @@
       <x:c r="H1" s="13"/>
       <x:c r="I1" s="13"/>
       <x:c r="J1" s="13"/>
+      <x:c r="K1" s="13"/>
+      <x:c r="L1" s="13"/>
+      <x:c r="M1" s="13"/>
+      <x:c r="N1" s="13"/>
+      <x:c r="O1" s="13"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str">
@@ -612,6 +627,11 @@
       <x:c r="H3" s="7"/>
       <x:c r="I3" s="7"/>
       <x:c r="J3" s="7"/>
+      <x:c r="K3" s="7"/>
+      <x:c r="L3" s="7"/>
+      <x:c r="M3" s="7"/>
+      <x:c r="N3" s="7"/>
+      <x:c r="O3" s="7"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
@@ -644,6 +664,21 @@
       <x:c r="J5" s="3" t="str">
         <x:v>Notas</x:v>
       </x:c>
+      <x:c r="K5" s="3" t="str">
+        <x:v>Dataverse estado</x:v>
+      </x:c>
+      <x:c r="L5" s="3" t="str">
+        <x:v>Ambiente</x:v>
+      </x:c>
+      <x:c r="M5" s="3" t="str">
+        <x:v>Target exacto</x:v>
+      </x:c>
+      <x:c r="N5" s="3" t="str">
+        <x:v>Gate live</x:v>
+      </x:c>
+      <x:c r="O5" s="3" t="str">
+        <x:v>Postcheck</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="str">
@@ -676,6 +711,21 @@
       <x:c r="J6" s="10" t="str">
         <x:v>Mesa viva para que nuevos hilos nazcan con contexto.</x:v>
       </x:c>
+      <x:c r="K6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="str">
@@ -708,6 +758,21 @@
       <x:c r="J7" s="10" t="str">
         <x:v>El conocimiento operativo queda promovible a canon, hito, tool o playbook.</x:v>
       </x:c>
+      <x:c r="K7" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L7" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M7" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N7" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O7" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="10" t="str">
@@ -740,6 +805,21 @@
       <x:c r="J8" s="10" t="str">
         <x:v>Validador read-only: archivos requeridos, mapas, links, xlsx y formulas.</x:v>
       </x:c>
+      <x:c r="K8" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L8" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M8" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N8" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O8" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="10" t="str">
@@ -772,6 +852,21 @@
       <x:c r="J9" s="10" t="str">
         <x:v>Incluye Resumen, Registro, Alertas y Listas.</x:v>
       </x:c>
+      <x:c r="K9" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L9" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M9" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N9" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O9" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="str">
@@ -804,6 +899,21 @@
       <x:c r="J10" s="10" t="str">
         <x:v>Gate local para cualquier trabajo Dataverse desde `PROJEC CDX`.</x:v>
       </x:c>
+      <x:c r="K10" s="10" t="str">
+        <x:v>metadata_only</x:v>
+      </x:c>
+      <x:c r="L10" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N10" s="10" t="str">
+        <x:v>cerrado</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="str">
+        <x:v>pendiente</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
@@ -836,6 +946,21 @@
       <x:c r="J11" s="10" t="str">
         <x:v>Dataverse sirve mejor como registro de bloqueos, decisiones y escaladas humanas que como inventario general.</x:v>
       </x:c>
+      <x:c r="K11" s="10" t="str">
+        <x:v>prepared_not_executed</x:v>
+      </x:c>
+      <x:c r="L11" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="M11" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N11" s="10" t="str">
+        <x:v>cerrado</x:v>
+      </x:c>
+      <x:c r="O11" s="10" t="str">
+        <x:v>pendiente</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
@@ -868,6 +993,21 @@
       <x:c r="J12" s="10" t="str">
         <x:v>El hilo queda navegable por capas, con detalle en hitos hijos.</x:v>
       </x:c>
+      <x:c r="K12" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L12" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M12" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N12" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O12" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="10" t="str">
@@ -900,6 +1040,21 @@
       <x:c r="J13" s="10" t="str">
         <x:v>Lista corta de pendientes vivos de `PROJEC CDX`.</x:v>
       </x:c>
+      <x:c r="K13" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L13" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M13" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N13" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O13" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="10" t="str">
@@ -931,6 +1086,21 @@
       </x:c>
       <x:c r="J14" s="10" t="str">
         <x:v>HECHO_VERIFICADO: revision GitHub live read-only completada.</x:v>
+      </x:c>
+      <x:c r="K14" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="L14" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="M14" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="N14" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="O14" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -944,6 +1114,11 @@
       <x:c r="H15" s="10"/>
       <x:c r="I15" s="10"/>
       <x:c r="J15" s="10"/>
+      <x:c r="K15" s="10"/>
+      <x:c r="L15" s="10"/>
+      <x:c r="M15" s="10"/>
+      <x:c r="N15" s="10"/>
+      <x:c r="O15" s="10"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="10"/>
@@ -956,6 +1131,11 @@
       <x:c r="H16" s="10"/>
       <x:c r="I16" s="10"/>
       <x:c r="J16" s="10"/>
+      <x:c r="K16" s="10"/>
+      <x:c r="L16" s="10"/>
+      <x:c r="M16" s="10"/>
+      <x:c r="N16" s="10"/>
+      <x:c r="O16" s="10"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="10"/>
@@ -968,6 +1148,11 @@
       <x:c r="H17" s="10"/>
       <x:c r="I17" s="10"/>
       <x:c r="J17" s="10"/>
+      <x:c r="K17" s="10"/>
+      <x:c r="L17" s="10"/>
+      <x:c r="M17" s="10"/>
+      <x:c r="N17" s="10"/>
+      <x:c r="O17" s="10"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="10"/>
@@ -980,6 +1165,11 @@
       <x:c r="H18" s="10"/>
       <x:c r="I18" s="10"/>
       <x:c r="J18" s="10"/>
+      <x:c r="K18" s="10"/>
+      <x:c r="L18" s="10"/>
+      <x:c r="M18" s="10"/>
+      <x:c r="N18" s="10"/>
+      <x:c r="O18" s="10"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="10"/>
@@ -992,6 +1182,11 @@
       <x:c r="H19" s="10"/>
       <x:c r="I19" s="10"/>
       <x:c r="J19" s="10"/>
+      <x:c r="K19" s="10"/>
+      <x:c r="L19" s="10"/>
+      <x:c r="M19" s="10"/>
+      <x:c r="N19" s="10"/>
+      <x:c r="O19" s="10"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="10"/>
@@ -1004,6 +1199,11 @@
       <x:c r="H20" s="10"/>
       <x:c r="I20" s="10"/>
       <x:c r="J20" s="10"/>
+      <x:c r="K20" s="10"/>
+      <x:c r="L20" s="10"/>
+      <x:c r="M20" s="10"/>
+      <x:c r="N20" s="10"/>
+      <x:c r="O20" s="10"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="10"/>
@@ -1016,6 +1216,11 @@
       <x:c r="H21" s="10"/>
       <x:c r="I21" s="10"/>
       <x:c r="J21" s="10"/>
+      <x:c r="K21" s="10"/>
+      <x:c r="L21" s="10"/>
+      <x:c r="M21" s="10"/>
+      <x:c r="N21" s="10"/>
+      <x:c r="O21" s="10"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="10"/>
@@ -1028,6 +1233,11 @@
       <x:c r="H22" s="10"/>
       <x:c r="I22" s="10"/>
       <x:c r="J22" s="10"/>
+      <x:c r="K22" s="10"/>
+      <x:c r="L22" s="10"/>
+      <x:c r="M22" s="10"/>
+      <x:c r="N22" s="10"/>
+      <x:c r="O22" s="10"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="10"/>
@@ -1040,6 +1250,11 @@
       <x:c r="H23" s="10"/>
       <x:c r="I23" s="10"/>
       <x:c r="J23" s="10"/>
+      <x:c r="K23" s="10"/>
+      <x:c r="L23" s="10"/>
+      <x:c r="M23" s="10"/>
+      <x:c r="N23" s="10"/>
+      <x:c r="O23" s="10"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="10"/>
@@ -1052,6 +1267,11 @@
       <x:c r="H24" s="10"/>
       <x:c r="I24" s="10"/>
       <x:c r="J24" s="10"/>
+      <x:c r="K24" s="10"/>
+      <x:c r="L24" s="10"/>
+      <x:c r="M24" s="10"/>
+      <x:c r="N24" s="10"/>
+      <x:c r="O24" s="10"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="10"/>
@@ -1064,6 +1284,11 @@
       <x:c r="H25" s="10"/>
       <x:c r="I25" s="10"/>
       <x:c r="J25" s="10"/>
+      <x:c r="K25" s="10"/>
+      <x:c r="L25" s="10"/>
+      <x:c r="M25" s="10"/>
+      <x:c r="N25" s="10"/>
+      <x:c r="O25" s="10"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="10"/>
@@ -1076,6 +1301,11 @@
       <x:c r="H26" s="10"/>
       <x:c r="I26" s="10"/>
       <x:c r="J26" s="10"/>
+      <x:c r="K26" s="10"/>
+      <x:c r="L26" s="10"/>
+      <x:c r="M26" s="10"/>
+      <x:c r="N26" s="10"/>
+      <x:c r="O26" s="10"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="10"/>
@@ -1088,6 +1318,11 @@
       <x:c r="H27" s="10"/>
       <x:c r="I27" s="10"/>
       <x:c r="J27" s="10"/>
+      <x:c r="K27" s="10"/>
+      <x:c r="L27" s="10"/>
+      <x:c r="M27" s="10"/>
+      <x:c r="N27" s="10"/>
+      <x:c r="O27" s="10"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="10"/>
@@ -1100,6 +1335,11 @@
       <x:c r="H28" s="10"/>
       <x:c r="I28" s="10"/>
       <x:c r="J28" s="10"/>
+      <x:c r="K28" s="10"/>
+      <x:c r="L28" s="10"/>
+      <x:c r="M28" s="10"/>
+      <x:c r="N28" s="10"/>
+      <x:c r="O28" s="10"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="10"/>
@@ -1112,6 +1352,11 @@
       <x:c r="H29" s="10"/>
       <x:c r="I29" s="10"/>
       <x:c r="J29" s="10"/>
+      <x:c r="K29" s="10"/>
+      <x:c r="L29" s="10"/>
+      <x:c r="M29" s="10"/>
+      <x:c r="N29" s="10"/>
+      <x:c r="O29" s="10"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="10"/>
@@ -1124,6 +1369,11 @@
       <x:c r="H30" s="10"/>
       <x:c r="I30" s="10"/>
       <x:c r="J30" s="10"/>
+      <x:c r="K30" s="10"/>
+      <x:c r="L30" s="10"/>
+      <x:c r="M30" s="10"/>
+      <x:c r="N30" s="10"/>
+      <x:c r="O30" s="10"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="10"/>
@@ -1136,6 +1386,11 @@
       <x:c r="H31" s="10"/>
       <x:c r="I31" s="10"/>
       <x:c r="J31" s="10"/>
+      <x:c r="K31" s="10"/>
+      <x:c r="L31" s="10"/>
+      <x:c r="M31" s="10"/>
+      <x:c r="N31" s="10"/>
+      <x:c r="O31" s="10"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="10"/>
@@ -1148,6 +1403,11 @@
       <x:c r="H32" s="10"/>
       <x:c r="I32" s="10"/>
       <x:c r="J32" s="10"/>
+      <x:c r="K32" s="10"/>
+      <x:c r="L32" s="10"/>
+      <x:c r="M32" s="10"/>
+      <x:c r="N32" s="10"/>
+      <x:c r="O32" s="10"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10"/>
@@ -1160,6 +1420,11 @@
       <x:c r="H33" s="10"/>
       <x:c r="I33" s="10"/>
       <x:c r="J33" s="10"/>
+      <x:c r="K33" s="10"/>
+      <x:c r="L33" s="10"/>
+      <x:c r="M33" s="10"/>
+      <x:c r="N33" s="10"/>
+      <x:c r="O33" s="10"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="10"/>
@@ -1172,6 +1437,11 @@
       <x:c r="H34" s="10"/>
       <x:c r="I34" s="10"/>
       <x:c r="J34" s="10"/>
+      <x:c r="K34" s="10"/>
+      <x:c r="L34" s="10"/>
+      <x:c r="M34" s="10"/>
+      <x:c r="N34" s="10"/>
+      <x:c r="O34" s="10"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="10"/>
@@ -1184,6 +1454,11 @@
       <x:c r="H35" s="10"/>
       <x:c r="I35" s="10"/>
       <x:c r="J35" s="10"/>
+      <x:c r="K35" s="10"/>
+      <x:c r="L35" s="10"/>
+      <x:c r="M35" s="10"/>
+      <x:c r="N35" s="10"/>
+      <x:c r="O35" s="10"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="10"/>
@@ -1196,6 +1471,11 @@
       <x:c r="H36" s="10"/>
       <x:c r="I36" s="10"/>
       <x:c r="J36" s="10"/>
+      <x:c r="K36" s="10"/>
+      <x:c r="L36" s="10"/>
+      <x:c r="M36" s="10"/>
+      <x:c r="N36" s="10"/>
+      <x:c r="O36" s="10"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="10"/>
@@ -1208,6 +1488,11 @@
       <x:c r="H37" s="10"/>
       <x:c r="I37" s="10"/>
       <x:c r="J37" s="10"/>
+      <x:c r="K37" s="10"/>
+      <x:c r="L37" s="10"/>
+      <x:c r="M37" s="10"/>
+      <x:c r="N37" s="10"/>
+      <x:c r="O37" s="10"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="10"/>
@@ -1220,6 +1505,11 @@
       <x:c r="H38" s="10"/>
       <x:c r="I38" s="10"/>
       <x:c r="J38" s="10"/>
+      <x:c r="K38" s="10"/>
+      <x:c r="L38" s="10"/>
+      <x:c r="M38" s="10"/>
+      <x:c r="N38" s="10"/>
+      <x:c r="O38" s="10"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="10"/>
@@ -1232,6 +1522,11 @@
       <x:c r="H39" s="10"/>
       <x:c r="I39" s="10"/>
       <x:c r="J39" s="10"/>
+      <x:c r="K39" s="10"/>
+      <x:c r="L39" s="10"/>
+      <x:c r="M39" s="10"/>
+      <x:c r="N39" s="10"/>
+      <x:c r="O39" s="10"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="10"/>
@@ -1244,6 +1539,11 @@
       <x:c r="H40" s="10"/>
       <x:c r="I40" s="10"/>
       <x:c r="J40" s="10"/>
+      <x:c r="K40" s="10"/>
+      <x:c r="L40" s="10"/>
+      <x:c r="M40" s="10"/>
+      <x:c r="N40" s="10"/>
+      <x:c r="O40" s="10"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="10"/>
@@ -1256,6 +1556,11 @@
       <x:c r="H41" s="10"/>
       <x:c r="I41" s="10"/>
       <x:c r="J41" s="10"/>
+      <x:c r="K41" s="10"/>
+      <x:c r="L41" s="10"/>
+      <x:c r="M41" s="10"/>
+      <x:c r="N41" s="10"/>
+      <x:c r="O41" s="10"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="10"/>
@@ -1268,6 +1573,11 @@
       <x:c r="H42" s="10"/>
       <x:c r="I42" s="10"/>
       <x:c r="J42" s="10"/>
+      <x:c r="K42" s="10"/>
+      <x:c r="L42" s="10"/>
+      <x:c r="M42" s="10"/>
+      <x:c r="N42" s="10"/>
+      <x:c r="O42" s="10"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="10"/>
@@ -1280,6 +1590,11 @@
       <x:c r="H43" s="10"/>
       <x:c r="I43" s="10"/>
       <x:c r="J43" s="10"/>
+      <x:c r="K43" s="10"/>
+      <x:c r="L43" s="10"/>
+      <x:c r="M43" s="10"/>
+      <x:c r="N43" s="10"/>
+      <x:c r="O43" s="10"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="10"/>
@@ -1292,6 +1607,11 @@
       <x:c r="H44" s="10"/>
       <x:c r="I44" s="10"/>
       <x:c r="J44" s="10"/>
+      <x:c r="K44" s="10"/>
+      <x:c r="L44" s="10"/>
+      <x:c r="M44" s="10"/>
+      <x:c r="N44" s="10"/>
+      <x:c r="O44" s="10"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="10"/>
@@ -1304,6 +1624,11 @@
       <x:c r="H45" s="10"/>
       <x:c r="I45" s="10"/>
       <x:c r="J45" s="10"/>
+      <x:c r="K45" s="10"/>
+      <x:c r="L45" s="10"/>
+      <x:c r="M45" s="10"/>
+      <x:c r="N45" s="10"/>
+      <x:c r="O45" s="10"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="10"/>
@@ -1316,6 +1641,11 @@
       <x:c r="H46" s="10"/>
       <x:c r="I46" s="10"/>
       <x:c r="J46" s="10"/>
+      <x:c r="K46" s="10"/>
+      <x:c r="L46" s="10"/>
+      <x:c r="M46" s="10"/>
+      <x:c r="N46" s="10"/>
+      <x:c r="O46" s="10"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="10"/>
@@ -1328,6 +1658,11 @@
       <x:c r="H47" s="10"/>
       <x:c r="I47" s="10"/>
       <x:c r="J47" s="10"/>
+      <x:c r="K47" s="10"/>
+      <x:c r="L47" s="10"/>
+      <x:c r="M47" s="10"/>
+      <x:c r="N47" s="10"/>
+      <x:c r="O47" s="10"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="10"/>
@@ -1340,6 +1675,11 @@
       <x:c r="H48" s="10"/>
       <x:c r="I48" s="10"/>
       <x:c r="J48" s="10"/>
+      <x:c r="K48" s="10"/>
+      <x:c r="L48" s="10"/>
+      <x:c r="M48" s="10"/>
+      <x:c r="N48" s="10"/>
+      <x:c r="O48" s="10"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="10"/>
@@ -1352,6 +1692,11 @@
       <x:c r="H49" s="10"/>
       <x:c r="I49" s="10"/>
       <x:c r="J49" s="10"/>
+      <x:c r="K49" s="10"/>
+      <x:c r="L49" s="10"/>
+      <x:c r="M49" s="10"/>
+      <x:c r="N49" s="10"/>
+      <x:c r="O49" s="10"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="10"/>
@@ -1364,6 +1709,11 @@
       <x:c r="H50" s="10"/>
       <x:c r="I50" s="10"/>
       <x:c r="J50" s="10"/>
+      <x:c r="K50" s="10"/>
+      <x:c r="L50" s="10"/>
+      <x:c r="M50" s="10"/>
+      <x:c r="N50" s="10"/>
+      <x:c r="O50" s="10"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="10"/>
@@ -1376,6 +1726,11 @@
       <x:c r="H51" s="10"/>
       <x:c r="I51" s="10"/>
       <x:c r="J51" s="10"/>
+      <x:c r="K51" s="10"/>
+      <x:c r="L51" s="10"/>
+      <x:c r="M51" s="10"/>
+      <x:c r="N51" s="10"/>
+      <x:c r="O51" s="10"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="10"/>
@@ -1388,6 +1743,11 @@
       <x:c r="H52" s="10"/>
       <x:c r="I52" s="10"/>
       <x:c r="J52" s="10"/>
+      <x:c r="K52" s="10"/>
+      <x:c r="L52" s="10"/>
+      <x:c r="M52" s="10"/>
+      <x:c r="N52" s="10"/>
+      <x:c r="O52" s="10"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="10"/>
@@ -1400,6 +1760,11 @@
       <x:c r="H53" s="10"/>
       <x:c r="I53" s="10"/>
       <x:c r="J53" s="10"/>
+      <x:c r="K53" s="10"/>
+      <x:c r="L53" s="10"/>
+      <x:c r="M53" s="10"/>
+      <x:c r="N53" s="10"/>
+      <x:c r="O53" s="10"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="10"/>
@@ -1412,6 +1777,11 @@
       <x:c r="H54" s="10"/>
       <x:c r="I54" s="10"/>
       <x:c r="J54" s="10"/>
+      <x:c r="K54" s="10"/>
+      <x:c r="L54" s="10"/>
+      <x:c r="M54" s="10"/>
+      <x:c r="N54" s="10"/>
+      <x:c r="O54" s="10"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="10"/>
@@ -1424,6 +1794,11 @@
       <x:c r="H55" s="10"/>
       <x:c r="I55" s="10"/>
       <x:c r="J55" s="10"/>
+      <x:c r="K55" s="10"/>
+      <x:c r="L55" s="10"/>
+      <x:c r="M55" s="10"/>
+      <x:c r="N55" s="10"/>
+      <x:c r="O55" s="10"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="10"/>
@@ -1436,6 +1811,11 @@
       <x:c r="H56" s="10"/>
       <x:c r="I56" s="10"/>
       <x:c r="J56" s="10"/>
+      <x:c r="K56" s="10"/>
+      <x:c r="L56" s="10"/>
+      <x:c r="M56" s="10"/>
+      <x:c r="N56" s="10"/>
+      <x:c r="O56" s="10"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="10"/>
@@ -1448,6 +1828,11 @@
       <x:c r="H57" s="10"/>
       <x:c r="I57" s="10"/>
       <x:c r="J57" s="10"/>
+      <x:c r="K57" s="10"/>
+      <x:c r="L57" s="10"/>
+      <x:c r="M57" s="10"/>
+      <x:c r="N57" s="10"/>
+      <x:c r="O57" s="10"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="10"/>
@@ -1460,6 +1845,11 @@
       <x:c r="H58" s="10"/>
       <x:c r="I58" s="10"/>
       <x:c r="J58" s="10"/>
+      <x:c r="K58" s="10"/>
+      <x:c r="L58" s="10"/>
+      <x:c r="M58" s="10"/>
+      <x:c r="N58" s="10"/>
+      <x:c r="O58" s="10"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="10"/>
@@ -1472,6 +1862,11 @@
       <x:c r="H59" s="10"/>
       <x:c r="I59" s="10"/>
       <x:c r="J59" s="10"/>
+      <x:c r="K59" s="10"/>
+      <x:c r="L59" s="10"/>
+      <x:c r="M59" s="10"/>
+      <x:c r="N59" s="10"/>
+      <x:c r="O59" s="10"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="10"/>
@@ -1484,6 +1879,11 @@
       <x:c r="H60" s="10"/>
       <x:c r="I60" s="10"/>
       <x:c r="J60" s="10"/>
+      <x:c r="K60" s="10"/>
+      <x:c r="L60" s="10"/>
+      <x:c r="M60" s="10"/>
+      <x:c r="N60" s="10"/>
+      <x:c r="O60" s="10"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="10"/>
@@ -1496,6 +1896,11 @@
       <x:c r="H61" s="10"/>
       <x:c r="I61" s="10"/>
       <x:c r="J61" s="10"/>
+      <x:c r="K61" s="10"/>
+      <x:c r="L61" s="10"/>
+      <x:c r="M61" s="10"/>
+      <x:c r="N61" s="10"/>
+      <x:c r="O61" s="10"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="10"/>
@@ -1508,6 +1913,11 @@
       <x:c r="H62" s="10"/>
       <x:c r="I62" s="10"/>
       <x:c r="J62" s="10"/>
+      <x:c r="K62" s="10"/>
+      <x:c r="L62" s="10"/>
+      <x:c r="M62" s="10"/>
+      <x:c r="N62" s="10"/>
+      <x:c r="O62" s="10"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="10"/>
@@ -1520,6 +1930,11 @@
       <x:c r="H63" s="10"/>
       <x:c r="I63" s="10"/>
       <x:c r="J63" s="10"/>
+      <x:c r="K63" s="10"/>
+      <x:c r="L63" s="10"/>
+      <x:c r="M63" s="10"/>
+      <x:c r="N63" s="10"/>
+      <x:c r="O63" s="10"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="10"/>
@@ -1532,6 +1947,11 @@
       <x:c r="H64" s="10"/>
       <x:c r="I64" s="10"/>
       <x:c r="J64" s="10"/>
+      <x:c r="K64" s="10"/>
+      <x:c r="L64" s="10"/>
+      <x:c r="M64" s="10"/>
+      <x:c r="N64" s="10"/>
+      <x:c r="O64" s="10"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="10"/>
@@ -1544,13 +1964,18 @@
       <x:c r="H65" s="10"/>
       <x:c r="I65" s="10"/>
       <x:c r="J65" s="10"/>
+      <x:c r="K65" s="10"/>
+      <x:c r="L65" s="10"/>
+      <x:c r="M65" s="10"/>
+      <x:c r="N65" s="10"/>
+      <x:c r="O65" s="10"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A3:J3"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A3:O3"/>
   </x:mergeCells>
-  <x:dataValidations count="3">
+  <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="C6:C65">
       <x:formula1>Listas!$A$3:$A$15</x:formula1>
     </x:dataValidation>
@@ -1560,10 +1985,22 @@
     <x:dataValidation type="list" sqref="F6:F65">
       <x:formula1>Listas!$C$3:$C$8</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="K6:K65">
+      <x:formula1>Listas!$E$3:$E$7</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L6:L65">
+      <x:formula1>Listas!$F$3:$F$6</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N6:N65">
+      <x:formula1>Listas!$G$3:$G$6</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="O6:O65">
+      <x:formula1>Listas!$H$3:$H$6</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76df418afd354a48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R375772591a7742aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1722,59 +2159,83 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
-        <x:v>ALR-006</x:v>
+        <x:v>ALR-008</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Media</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>hitos</x:v>
+        <x:v>dataverse</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>auditar_child_classification_pending</x:v>
+        <x:v>metadata_only_requires_postcheck</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Clasificar hijos de Auditar antes de mover, borrar, promover o escribir.</x:v>
+        <x:v>No cerrar metadata_only sin postcheck visible y evidencia local suficiente.</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>operativa/TODO_20260615.md</x:v>
+        <x:v>dataverse/PLAN_SEGUNDA_PASADA.md</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
+        <x:v>ALR-009</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>dataverse</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>prepared_not_executed_requires_owner</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>No dejar prepared_not_executed sin owner asignado y target no ambiguo.</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>dataverse/PLAN_SEGUNDA_PASADA.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="10" t="str">
+        <x:v>ALR-006</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>Media</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>hitos</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>auditar_child_classification_pending</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>Clasificar hijos de Auditar antes de mover, borrar, promover o escribir.</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="str">
+        <x:v>operativa/TODO_20260615.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="10" t="str">
         <x:v>ALR-007</x:v>
       </x:c>
-      <x:c r="B12" s="10" t="str">
+      <x:c r="B14" s="10" t="str">
         <x:v>Media</x:v>
       </x:c>
-      <x:c r="C12" s="10" t="str">
+      <x:c r="C14" s="10" t="str">
         <x:v>github</x:v>
       </x:c>
-      <x:c r="D12" s="10" t="str">
+      <x:c r="D14" s="10" t="str">
         <x:v>github_write_requires_atomic_order</x:v>
       </x:c>
-      <x:c r="E12" s="10" t="str">
+      <x:c r="E14" s="10" t="str">
         <x:v>No mergear, comentar, pushear ni modificar PRs sin target exacto, owner, rollback, postcheck y evidencia.</x:v>
       </x:c>
-      <x:c r="F12" s="10" t="str">
+      <x:c r="F14" s="10" t="str">
         <x:v>outputs/live_repo_review_20260615/READBACK.md</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="10"/>
-      <x:c r="B13" s="10"/>
-      <x:c r="C13" s="10"/>
-      <x:c r="D13" s="10"/>
-      <x:c r="E13" s="10"/>
-      <x:c r="F13" s="10"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="10"/>
-      <x:c r="B14" s="10"/>
-      <x:c r="C14" s="10"/>
-      <x:c r="D14" s="10"/>
-      <x:c r="E14" s="10"/>
-      <x:c r="F14" s="10"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="10"/>
@@ -1956,7 +2417,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd886678abca54277"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca3878ba6ab4c87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1969,6 +2430,10 @@
     <x:col min="2" max="2" width="22.5" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22.5" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1992,6 +2457,18 @@
       <x:c r="D2" s="3" t="str">
         <x:v>Severidades</x:v>
       </x:c>
+      <x:c r="E2" s="3" t="str">
+        <x:v>Dataverse estados</x:v>
+      </x:c>
+      <x:c r="F2" s="3" t="str">
+        <x:v>Ambientes</x:v>
+      </x:c>
+      <x:c r="G2" s="3" t="str">
+        <x:v>Gate live</x:v>
+      </x:c>
+      <x:c r="H2" s="3" t="str">
+        <x:v>Postcheck</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
@@ -2006,6 +2483,18 @@
       <x:c r="D3" s="10" t="str">
         <x:v>Info</x:v>
       </x:c>
+      <x:c r="E3" s="10" t="str">
+        <x:v>local_evidence</x:v>
+      </x:c>
+      <x:c r="F3" s="10" t="str">
+        <x:v>local</x:v>
+      </x:c>
+      <x:c r="G3" s="10" t="str">
+        <x:v>cerrado</x:v>
+      </x:c>
+      <x:c r="H3" s="10" t="str">
+        <x:v>pendiente</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="str">
@@ -2020,6 +2509,18 @@
       <x:c r="D4" s="10" t="str">
         <x:v>Baja</x:v>
       </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>metadata_only</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="str">
+        <x:v>metadata_only</x:v>
+      </x:c>
+      <x:c r="G4" s="10" t="str">
+        <x:v>abierto</x:v>
+      </x:c>
+      <x:c r="H4" s="10" t="str">
+        <x:v>ok</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="10" t="str">
@@ -2034,6 +2535,18 @@
       <x:c r="D5" s="10" t="str">
         <x:v>Media</x:v>
       </x:c>
+      <x:c r="E5" s="10" t="str">
+        <x:v>prepared_not_executed</x:v>
+      </x:c>
+      <x:c r="F5" s="10" t="str">
+        <x:v>live</x:v>
+      </x:c>
+      <x:c r="G5" s="10" t="str">
+        <x:v>n/a</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="str">
+        <x:v>n/a</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="10" t="str">
@@ -2048,6 +2561,18 @@
       <x:c r="D6" s="10" t="str">
         <x:v>Alta</x:v>
       </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>live_rows_confirmed</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
+      <x:c r="H6" s="10" t="str">
+        <x:v>NO_APLICA</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="10" t="str">
@@ -2060,6 +2585,12 @@
         <x:v>Cerrado</x:v>
       </x:c>
       <x:c r="D7" s="10"/>
+      <x:c r="E7" s="10" t="str">
+        <x:v>blocked</x:v>
+      </x:c>
+      <x:c r="F7" s="10"/>
+      <x:c r="G7" s="10"/>
+      <x:c r="H7" s="10"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="10" t="str">
@@ -2072,6 +2603,10 @@
         <x:v>Versionado</x:v>
       </x:c>
       <x:c r="D8" s="10"/>
+      <x:c r="E8" s="10"/>
+      <x:c r="F8" s="10"/>
+      <x:c r="G8" s="10"/>
+      <x:c r="H8" s="10"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="10" t="str">
@@ -2082,6 +2617,10 @@
       </x:c>
       <x:c r="C9" s="10"/>
       <x:c r="D9" s="10"/>
+      <x:c r="E9" s="10"/>
+      <x:c r="F9" s="10"/>
+      <x:c r="G9" s="10"/>
+      <x:c r="H9" s="10"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="str">
@@ -2092,6 +2631,10 @@
       </x:c>
       <x:c r="C10" s="10"/>
       <x:c r="D10" s="10"/>
+      <x:c r="E10" s="10"/>
+      <x:c r="F10" s="10"/>
+      <x:c r="G10" s="10"/>
+      <x:c r="H10" s="10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
@@ -2102,6 +2645,10 @@
       </x:c>
       <x:c r="C11" s="10"/>
       <x:c r="D11" s="10"/>
+      <x:c r="E11" s="10"/>
+      <x:c r="F11" s="10"/>
+      <x:c r="G11" s="10"/>
+      <x:c r="H11" s="10"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
@@ -2110,6 +2657,10 @@
       <x:c r="B12" s="10"/>
       <x:c r="C12" s="10"/>
       <x:c r="D12" s="10"/>
+      <x:c r="E12" s="10"/>
+      <x:c r="F12" s="10"/>
+      <x:c r="G12" s="10"/>
+      <x:c r="H12" s="10"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="10" t="str">
@@ -2118,6 +2669,10 @@
       <x:c r="B13" s="10"/>
       <x:c r="C13" s="10"/>
       <x:c r="D13" s="10"/>
+      <x:c r="E13" s="10"/>
+      <x:c r="F13" s="10"/>
+      <x:c r="G13" s="10"/>
+      <x:c r="H13" s="10"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="10" t="str">
@@ -2126,6 +2681,10 @@
       <x:c r="B14" s="10"/>
       <x:c r="C14" s="10"/>
       <x:c r="D14" s="10"/>
+      <x:c r="E14" s="10"/>
+      <x:c r="F14" s="10"/>
+      <x:c r="G14" s="10"/>
+      <x:c r="H14" s="10"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="10" t="str">
@@ -2134,6 +2693,10 @@
       <x:c r="B15" s="10"/>
       <x:c r="C15" s="10"/>
       <x:c r="D15" s="10"/>
+      <x:c r="E15" s="10"/>
+      <x:c r="F15" s="10"/>
+      <x:c r="G15" s="10"/>
+      <x:c r="H15" s="10"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>